<commit_message>
Added week 4 Prompt Engineering
</commit_message>
<xml_diff>
--- a/AI Audit Log_DE190499.xlsx
+++ b/AI Audit Log_DE190499.xlsx
@@ -8,21 +8,22 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\FPT Uni\Major5\SWP\ai-audit-log-btuejan11\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2607CF9-6D7F-4B07-801B-7DAFD9517A52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C588B66-48B6-4E41-9D06-9AD1EBAFA3E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet 2" sheetId="2" r:id="rId2"/>
-    <sheet name="Sheet3" sheetId="4" r:id="rId3"/>
+    <sheet name="Week 1" sheetId="1" r:id="rId1"/>
+    <sheet name="Week 2" sheetId="2" r:id="rId2"/>
+    <sheet name="Week 3" sheetId="5" r:id="rId3"/>
+    <sheet name="Week 4" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="125">
   <si>
     <t>STT (Entry #)</t>
   </si>
@@ -345,16 +346,174 @@
   <si>
     <t>Cần xác định định hướng thương hiệu và visual identity cho AuraSpa trước khi bắt đầu thiết kế bất kỳ màn hình nào</t>
   </si>
+  <si>
+    <t>Mở rộng Chi tiết</t>
+  </si>
+  <si>
+    <t>UC-10: Đặt Lịch Hẹn
+Luồng Chính</t>
+  </si>
+  <si>
+    <t>Luồng tuyến tính thiếu logic xác thực, kiểm tra trạng thái hệ thống. Cần kiểm tra tính khả dụng thực tế, ngăn chặn đặt quá giới hạn (BR-19), cân bằng tải kỹ thuật viên (BR-20), tích hợp discount (UC-14).</t>
+  </si>
+  <si>
+    <t>Mở rộng Luồng Chính 10→16 bước. Mỗi bước: hệ thống kiểm tra gì (tên trường, ràng buộc), tích hợp với UCs/BRs khác, xử lý lỗi. Tập trung phase xác nhận (tính toán giá, xác thực discount, xác nhận).</t>
+  </si>
+  <si>
+    <t>16 bước chi tiết:
+• Bước 5a-5c: Kiểm tra khe trống, booking đồng thời, xác thực chi nhánh
+• Bước 7a-7b: Validate discount API, tính toán lại giá
+• Bước 9-10: Tạo lịch hẹn, kích hoạt UC-38
+✓ Thêm: Kiểm tra trạng thái Đóng cửa tạm thời (BR-46)
+✓ Xử lý race condition với re-validation</t>
+  </si>
+  <si>
+    <t>Phát hiện Exception</t>
+  </si>
+  <si>
+    <t>UC-24: Tạo Hóa đơn
+Mở rộng Exception &amp; BR</t>
+  </si>
+  <si>
+    <t>Chỉ 2 exception; thiếu gói nhiều buổi, hoàn tiền từng phần, tính hoa hồng kỹ thuật viên, VAT (Việt Nam), hủy hóa đơn, tích hợp tồn kho (UC-30).</t>
+  </si>
+  <si>
+    <t>8 exception flow: deduction nhiều buổi, hoàn tiền, tính commission, lỗi thanh toán, thiếu tồn kho, ngăn trùng lập, áp dụng VAT, chuyển quyền thanh toán. Cộng 5 BR mới cho hóa đơn.</t>
+  </si>
+  <si>
+    <t>8 flow (E1-E8):
+• E3: Nhiều buổi → trừ remaining_sessions
+• E5: Thiếu tồn kho → ghi log, cho phép tạo
+• E7: Áp dụng VAT → thêm dòng, tính vào sổ
++ 5 BR: Tính bất biến, Deduction, Commission, Hủy
+✓ Phát hiện: Commission không có trong spec gốc</t>
+  </si>
+  <si>
+    <t>Tinh chỉnh Luồng Thay thế</t>
+  </si>
+  <si>
+    <t>UC-38: Gửi Thông báo
+Kênh &amp; Độ tin cậy</t>
+  </si>
+  <si>
+    <t>Giả định 1 kênh. Thiếu logic đa kênh (email/SMS/push), bản địa hóa ngôn ngữ, kiểm soát tần suất, failover nhà cung cấp, throttling khối lượng, versioning template.</t>
+  </si>
+  <si>
+    <t>7 luồng thay thế: chọn kênh đa (logic ưu tiên), ngôn ngữ, kiểm soát tần suất (max 2 reminder), failover (retry logic), throttling (50/giây), versioning template.</t>
+  </si>
+  <si>
+    <t>7 flow (2.1-2.7):
+• 2.1: Logic chọn kênh + fallback
+• 2.4: Retry failover 5-giây, cảnh báo admin
+• 2.5: Message queue + batch worker (50/sec)
++ 2 BR: Versioning, Throttling
+✓ Thêm: message_queue architecture, failover</t>
+  </si>
+  <si>
+    <t>Làm Rõ Điều kiện Trước</t>
+  </si>
+  <si>
+    <t>UC-27: Cấu hình Khe Thời gian
+Dependencies &amp; Constraints</t>
+  </si>
+  <si>
+    <t>Điều kiện trước mơ hồ: scope access control không rõ, phương thức tạo khe không định nghĩa, dependency schedule thiếu, constraint validation vắng, impact cấu hình trên appointment hiện tại mờ.</t>
+  </si>
+  <si>
+    <t>Chi tiết điều kiện trước: access control (chỉ chi nhánh mình?), dependencies (khe pre-created vs. dynamic), constraint validation (min/max concurrent), impact appointment hiện tại (BR-40), timing postcondition.</t>
+  </si>
+  <si>
+    <t>Điều kiện trước mở rộng:
+• Access: BM chỉ config chi nhánh mình
+• Khe: Cấu trúc pre-created (start, end, duration)
+• Ràng buộc: 1≤concurrent≤active_tech, duration≥min_service
+• Impact: Config từ mai, hôm nay không ảnh hưởng
+✓ Phát hiện: Pre-created vs. dynamic ảnh hưởng kiến trúc</t>
+  </si>
+  <si>
+    <t>Ưu tiên &amp; Tác động</t>
+  </si>
+  <si>
+    <t>UC-29: Giải quyết Khiếu nại
+SLA &amp; Framework Escalation</t>
+  </si>
+  <si>
+    <t>Thiếu taxonomy khiếu nại, mục tiêu SLA, tiêu chí escalation, giới hạn tài chính, liên kết KPI, chiến lược giữ khách, xử lý VIP.</t>
+  </si>
+  <si>
+    <t>8 danh mục khiếu nại → mapping priority + SLA (P1/P2/P3), resolution actions (hoàn tiền/comp limits), escalation rules (khi nào→Owner), tracking financial impact, staff/branch KPI.</t>
+  </si>
+  <si>
+    <t>8 danh mục (Vệ sinh, Billing, Chất lượng, Nhân viên, Cơ sở, Quyền riêng tư, Dị ứng, Feedback) → P1/P2/P3
+SLA: P1&lt;1h ack/24h resolve, P2&lt;8h ack/3d, P3&lt;24h ack/7d
+Escalation: P1, public, comp&gt;300k, VIP, 3+ khiếu nại/6th → Owner
++ 9 BR (BR-62-70)
+✓ Chuyển UC-29 thành KPI driver chiến lược</t>
+  </si>
+  <si>
+    <t>✓ Cải tiến: Luồng giờ đã developer-ready, có tên table, trường cụ thể
+✓ Phát hiện: Thiếu kiểm tra Temporarily Closed (BR-46) → Thêm
+✓ Điều chỉnh: Bước 6 gốc (2 concern) → Tách thành atomic steps
+⚠ Quyết định: Concurrent booking check TRƯỚC hiển thị (pessimistic) hay chỉ lúc confirm (optimistic)?
+  → CHỌN: Optimistic locking step 5c + re-validate step 8 để catch race condition
+✓ THÊM: Explicit error handling path cho mỗi validation failure
+PHẢN LOẠI: UC-10 là transaction-critical, cần detailed validation logic</t>
+  </si>
+  <si>
+    <t>✓ PHÁT HIỆN LỚN: UC-24 không đầy đủ – thiếu multi-session &amp; commission tracking
+✓ THÊM: E3 (Multi-session), E5 (Inventory shortage), E7 (VAT) – quan trọng cho spa VN
+✓ LIÊN KẾT TẠO: UC-24 giờ explicit connect tới UC-30 (Inventory) &amp; staff payroll concerns
+⚠ QUYẾT ĐỊNH: Technician commission là system-wide concern → có thể cần UC-39 "Calculate Staff Commission &amp; Payroll"
+✓ COMPLIANCE: BR-57-BR-61 cover Vietnam tax &amp; spa industry invoice requirements
+PHẢN LOẠI: Original UC-24 quá đơn giản; mở rộng này hỗ trợ real spa business operations</t>
+  </si>
+  <si>
+    <t>✓ CRITICAL ADDITION: Alt Flow 2.4 &amp; 2.5 address production-grade reliability (failover, throttling)
+✓ PHÁT HIỆN: Original UC-38 assume single channel; reality cần multi-channel logic + fallback
+✓ CONCERN MỚI: Notification template versioning là requirement chưa capture
+⚠ ARCHITECTURE IMPACT: Cần design message_queue table &amp; background worker service
+✓ COMPLIANCE: BR-54 (SMS opt-out) giờ integrate vào full channel selection logic
+PHẢN LOẠI: UC-38 tăng từ 3 thành 8+ flows; complex hơn initial spec
+NEXT STEP: Có thể cần UC-39 "Manage Notification Preferences &amp; Templates" (Owner/Manager config)</t>
+  </si>
+  <si>
+    <t>✓ CLARITY: Preconditions giờ explicit define access control, data dependencies, timeline
+✓ PHÁT HIỆN: Assumption slots pre-created (không dynamically generated) – important cho design
+✓ CONSTRAINT ADDED: max_concurrent_bookings không thể exceed active technician count – prevent overbooking
+⚠ COMPLEXITY: Slot structure (pre-created vs. dynamic) affect entire booking system architecture
+✓ TIMING CLARIFICATION: Config changes apply từ next day, không immediately – prevent race conditions
+PHẢN LOẠI: UC-27 actually configuration management UC với significant dependencies trên UC-21, UC-26, real-time slot availability
+NEXT STEP: Create data model cho booking_slot_config &amp; time_slot tables</t>
+  </si>
+  <si>
+    <t>✓ MAJOR EXPANSION: UC-29 tăng từ simple complaint resolution → comprehensive customer service &amp; retention strategy
+✓ CATEGORIES DEFINED: 8 categories with severity/priority mapping → consistent handling across branches
+✓ FINANCIAL CONTROLS: Compensation limits (BR-64) prevent BM over-committing refunds; Owner maintain financial control
+✓ KPI INTEGRATION: Complaints giờ tied to staff performance (retraining triggers), branch ratings (Owner visibility), customer retention
+✓ ESCALATION LOGIC: Clear rules prevent trivial complaints reaching Owner while ensuring critical ones do
+✓ DATA QUALITY: Immutable audit trail (BR-70) support regulatory compliance &amp; dispute resolution
+⚠ NEW CONCERN: Follow-up satisfaction survey (UC-38 extension) tạo feedback loop; need new survey UC or extend UC-38
+⚠ WORKFLOW ADDED: "Risky Customer" detection &amp; VIP prioritization add complexity
+PHẢN LOẠI: UC-29 giờ strategic KPI driver, không chỉ reactive issue handler. Impact Owner dashboards, staff metrics, customer retention
+NEXT STEP: Design complaint dashboard cho Owner showing trends, escalations, staff performance; integrate with UC-31</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -398,6 +557,12 @@
     <font>
       <sz val="9"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="major"/>
     </font>
   </fonts>
   <fills count="3">
@@ -468,43 +633,48 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1" xr:uid="{679B5E49-DA20-4155-934C-81DD4CB35B43}"/>
+    <cellStyle name="Normal 3" xfId="2" xr:uid="{31554C69-3A9C-4497-AEBA-DA8560C4FB23}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1216,6 +1386,277 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{94319FF9-09DD-4364-854F-EE2EC40DD129}">
+  <dimension ref="A1:G11"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="7" style="9" customWidth="1"/>
+    <col min="2" max="2" width="18" style="9" customWidth="1"/>
+    <col min="3" max="3" width="22" style="9" customWidth="1"/>
+    <col min="4" max="4" width="30" style="9" customWidth="1"/>
+    <col min="5" max="7" width="38" style="9" customWidth="1"/>
+    <col min="8" max="16384" width="8.88671875" style="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="G1" s="8" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="120" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="B2" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="C2" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="D2" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="E2" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="F2" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="G2" s="11" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="120" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="B3" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="C3" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="D3" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="E3" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="F3" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="G3" s="11" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="120" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="B4" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="D4" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="E4" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="F4" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="G4" s="11" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="120" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="B5" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="C5" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="D5" s="11" t="s">
+        <v>53</v>
+      </c>
+      <c r="E5" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="F5" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="G5" s="11" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="120" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="B6" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="D6" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="E6" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="F6" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="G6" s="11" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="120" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="B7" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="C7" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="D7" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="E7" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="F7" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="G7" s="11" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="120" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="B8" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="C8" s="11" t="s">
+        <v>70</v>
+      </c>
+      <c r="D8" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="E8" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="F8" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="G8" s="11" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="120" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="10" t="s">
+        <v>75</v>
+      </c>
+      <c r="B9" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="C9" s="11" t="s">
+        <v>76</v>
+      </c>
+      <c r="D9" s="11" t="s">
+        <v>77</v>
+      </c>
+      <c r="E9" s="11" t="s">
+        <v>78</v>
+      </c>
+      <c r="F9" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="G9" s="11" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="120" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="B10" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="C10" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="D10" s="11" t="s">
+        <v>83</v>
+      </c>
+      <c r="E10" s="11" t="s">
+        <v>84</v>
+      </c>
+      <c r="F10" s="11" t="s">
+        <v>85</v>
+      </c>
+      <c r="G10" s="11" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="120" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="10" t="s">
+        <v>87</v>
+      </c>
+      <c r="B11" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="C11" s="11" t="s">
+        <v>89</v>
+      </c>
+      <c r="D11" s="11" t="s">
+        <v>90</v>
+      </c>
+      <c r="E11" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="F11" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="G11" s="11" t="s">
+        <v>93</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8095962D-6AA5-44B9-881D-99D43448B400}">
   <dimension ref="A1:G11"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
@@ -1252,234 +1693,164 @@
       </c>
     </row>
     <row r="2" spans="1:7" ht="120" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="10" t="s">
+      <c r="A2" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="B2" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="C2" s="11" t="s">
-        <v>34</v>
-      </c>
-      <c r="D2" s="11" t="s">
-        <v>94</v>
-      </c>
-      <c r="E2" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="F2" s="11" t="s">
-        <v>36</v>
-      </c>
-      <c r="G2" s="11" t="s">
-        <v>37</v>
+      <c r="B2" s="12" t="s">
+        <v>95</v>
+      </c>
+      <c r="C2" s="12" t="s">
+        <v>96</v>
+      </c>
+      <c r="D2" s="12" t="s">
+        <v>97</v>
+      </c>
+      <c r="E2" s="12" t="s">
+        <v>98</v>
+      </c>
+      <c r="F2" s="12" t="s">
+        <v>99</v>
+      </c>
+      <c r="G2" s="12" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="120" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="10" t="s">
+      <c r="A3" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="B3" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="C3" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="D3" s="11" t="s">
-        <v>41</v>
-      </c>
-      <c r="E3" s="11" t="s">
-        <v>42</v>
-      </c>
-      <c r="F3" s="11" t="s">
-        <v>43</v>
-      </c>
-      <c r="G3" s="11" t="s">
-        <v>44</v>
+      <c r="B3" s="12" t="s">
+        <v>100</v>
+      </c>
+      <c r="C3" s="12" t="s">
+        <v>101</v>
+      </c>
+      <c r="D3" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="E3" s="12" t="s">
+        <v>103</v>
+      </c>
+      <c r="F3" s="12" t="s">
+        <v>104</v>
+      </c>
+      <c r="G3" s="12" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="120" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="10" t="s">
+      <c r="A4" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="B4" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="C4" s="11" t="s">
-        <v>46</v>
-      </c>
-      <c r="D4" s="11" t="s">
-        <v>47</v>
-      </c>
-      <c r="E4" s="11" t="s">
-        <v>48</v>
-      </c>
-      <c r="F4" s="11" t="s">
-        <v>49</v>
-      </c>
-      <c r="G4" s="11" t="s">
-        <v>50</v>
+      <c r="B4" s="12" t="s">
+        <v>105</v>
+      </c>
+      <c r="C4" s="12" t="s">
+        <v>106</v>
+      </c>
+      <c r="D4" s="12" t="s">
+        <v>107</v>
+      </c>
+      <c r="E4" s="12" t="s">
+        <v>108</v>
+      </c>
+      <c r="F4" s="12" t="s">
+        <v>109</v>
+      </c>
+      <c r="G4" s="12" t="s">
+        <v>122</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="120" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="10" t="s">
+      <c r="A5" s="12" t="s">
         <v>51</v>
       </c>
-      <c r="B5" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="C5" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="D5" s="11" t="s">
-        <v>53</v>
-      </c>
-      <c r="E5" s="11" t="s">
-        <v>54</v>
-      </c>
-      <c r="F5" s="11" t="s">
-        <v>55</v>
-      </c>
-      <c r="G5" s="11" t="s">
-        <v>56</v>
+      <c r="B5" s="12" t="s">
+        <v>110</v>
+      </c>
+      <c r="C5" s="12" t="s">
+        <v>111</v>
+      </c>
+      <c r="D5" s="12" t="s">
+        <v>112</v>
+      </c>
+      <c r="E5" s="12" t="s">
+        <v>113</v>
+      </c>
+      <c r="F5" s="12" t="s">
+        <v>114</v>
+      </c>
+      <c r="G5" s="12" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="120" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="10" t="s">
+      <c r="A6" s="12" t="s">
         <v>57</v>
       </c>
-      <c r="B6" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="C6" s="11" t="s">
-        <v>58</v>
-      </c>
-      <c r="D6" s="11" t="s">
-        <v>59</v>
-      </c>
-      <c r="E6" s="11" t="s">
-        <v>60</v>
-      </c>
-      <c r="F6" s="11" t="s">
-        <v>61</v>
-      </c>
-      <c r="G6" s="11" t="s">
-        <v>62</v>
+      <c r="B6" s="12" t="s">
+        <v>115</v>
+      </c>
+      <c r="C6" s="12" t="s">
+        <v>116</v>
+      </c>
+      <c r="D6" s="12" t="s">
+        <v>117</v>
+      </c>
+      <c r="E6" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="F6" s="12" t="s">
+        <v>119</v>
+      </c>
+      <c r="G6" s="12" t="s">
+        <v>124</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="120" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="10" t="s">
-        <v>63</v>
-      </c>
-      <c r="B7" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="C7" s="11" t="s">
-        <v>64</v>
-      </c>
-      <c r="D7" s="11" t="s">
-        <v>65</v>
-      </c>
-      <c r="E7" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="F7" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="G7" s="11" t="s">
-        <v>68</v>
-      </c>
+      <c r="A7" s="10"/>
+      <c r="B7" s="11"/>
+      <c r="C7" s="11"/>
+      <c r="D7" s="11"/>
+      <c r="E7" s="11"/>
+      <c r="F7" s="11"/>
+      <c r="G7" s="11"/>
     </row>
     <row r="8" spans="1:7" ht="120" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="10" t="s">
-        <v>69</v>
-      </c>
-      <c r="B8" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="C8" s="11" t="s">
-        <v>70</v>
-      </c>
-      <c r="D8" s="11" t="s">
-        <v>71</v>
-      </c>
-      <c r="E8" s="11" t="s">
-        <v>72</v>
-      </c>
-      <c r="F8" s="11" t="s">
-        <v>73</v>
-      </c>
-      <c r="G8" s="11" t="s">
-        <v>74</v>
-      </c>
+      <c r="A8" s="10"/>
+      <c r="B8" s="11"/>
+      <c r="C8" s="11"/>
+      <c r="D8" s="11"/>
+      <c r="E8" s="11"/>
+      <c r="F8" s="11"/>
+      <c r="G8" s="11"/>
     </row>
     <row r="9" spans="1:7" ht="120" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="10" t="s">
-        <v>75</v>
-      </c>
-      <c r="B9" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="C9" s="11" t="s">
-        <v>76</v>
-      </c>
-      <c r="D9" s="11" t="s">
-        <v>77</v>
-      </c>
-      <c r="E9" s="11" t="s">
-        <v>78</v>
-      </c>
-      <c r="F9" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="G9" s="11" t="s">
-        <v>80</v>
-      </c>
+      <c r="A9" s="10"/>
+      <c r="B9" s="11"/>
+      <c r="C9" s="11"/>
+      <c r="D9" s="11"/>
+      <c r="E9" s="11"/>
+      <c r="F9" s="11"/>
+      <c r="G9" s="11"/>
     </row>
     <row r="10" spans="1:7" ht="120" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="10" t="s">
-        <v>81</v>
-      </c>
-      <c r="B10" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="C10" s="11" t="s">
-        <v>82</v>
-      </c>
-      <c r="D10" s="11" t="s">
-        <v>83</v>
-      </c>
-      <c r="E10" s="11" t="s">
-        <v>84</v>
-      </c>
-      <c r="F10" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="G10" s="11" t="s">
-        <v>86</v>
-      </c>
+      <c r="A10" s="10"/>
+      <c r="B10" s="11"/>
+      <c r="C10" s="11"/>
+      <c r="D10" s="11"/>
+      <c r="E10" s="11"/>
+      <c r="F10" s="11"/>
+      <c r="G10" s="11"/>
     </row>
     <row r="11" spans="1:7" ht="120" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="10" t="s">
-        <v>87</v>
-      </c>
-      <c r="B11" s="11" t="s">
-        <v>88</v>
-      </c>
-      <c r="C11" s="11" t="s">
-        <v>89</v>
-      </c>
-      <c r="D11" s="11" t="s">
-        <v>90</v>
-      </c>
-      <c r="E11" s="11" t="s">
-        <v>91</v>
-      </c>
-      <c r="F11" s="11" t="s">
-        <v>92</v>
-      </c>
-      <c r="G11" s="11" t="s">
-        <v>93</v>
-      </c>
+      <c r="A11" s="10"/>
+      <c r="B11" s="11"/>
+      <c r="C11" s="11"/>
+      <c r="D11" s="11"/>
+      <c r="E11" s="11"/>
+      <c r="F11" s="11"/>
+      <c r="G11" s="11"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>